<commit_message>
feat: implement kitchen security system firmware with multi-sensor integration and reporting documentation
</commit_message>
<xml_diff>
--- a/Docs/SE190732_NgoGiaLong_AI_AuditLog_IOT102.xlsx
+++ b/Docs/SE190732_NgoGiaLong_AI_AuditLog_IOT102.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Semester 4\IOT102\iot-kitchen-security-system\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4356D88-09EB-4C2F-B04D-A6CE4148C14A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A13934B1-A035-4310-9CD9-8770B1206410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="161">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -96,9 +96,6 @@
   </si>
   <si>
     <t>Medium</t>
-  </si>
-  <si>
-    <t>[Add more...]</t>
   </si>
   <si>
     <t>CORE PROMPTS DISTRIBUTION BY DTC COMPONENT</t>
@@ -735,6 +732,44 @@
   <si>
     <t>https://docs.google.com/document/d/1_rVpJ0FGlCmkMVqam7iwtbF_toUpBtAB/edit?usp=sharing&amp;ouid=104267734760244325738&amp;rtpof=true&amp;sd=true</t>
   </si>
+  <si>
+    <t>Sau đợt đánh giá ở tuần thứ 7, tôi nhận thấy dự án IoT của mình gặp một số vấn đề về yêu cầu và tài liệu. Các tài liệu ban đầu còn rời rạc: có phần tập trung vào phần cứng, có phần mô tả các ý tưởng về tính năng cảnh báo, trong khi những phần khác lại chưa xác định rõ phạm vi dự án hay định hướng hiện tại của hệ thống. Từ kiến ​​thức trong môn học SWR, tôi hiểu rằng một hệ thống bài bản cần có tài liệu đặc tả yêu cầu (SRS) để làm rõ chức năng hệ thống, những gì hệ thống không thực hiện, ý nghĩa của từng biến số, cũng như cách các tác nhân AI trong tương lai cần hiểu bối cảnh dự án trước khi đưa ra hỗ trợ. Do đó, tôi quyết định không chỉ viết lại tài liệu SRS theo chuẩn chuyên nghiệp hơn, mà còn rà soát lại các tài liệu gốc để xem xét liệu những ý tưởng trước đó có còn phù hợp hay không sau đợt đánh giá tuần thứ 7.</t>
+  </si>
+  <si>
+    <t>After the week 7 review, I found that my IoT anti-theft project documents are fragmented and some earlier ideas may no longer match the current project direction. Based on what I learned from SWR, please help me reassess the old documents and rebuild the project requirements into a clear SRS. The SRS should define the system scope, removed scope, version history, agent rules, functional requirements, business rules, Cloud Variables, dashboards and acceptance scenarios. Do not simply rewrite the old content, and do not invent new modules without confirmation.</t>
+  </si>
+  <si>
+    <t>AI đã đề xuất coi công việc này là một đợt đánh giá lại các yêu cầu thay vì chỉ đơn thuần là viết lại tài liệu. AI đã hỗ trợ sắp xếp các ý tưởng rời rạc thành một tài liệu chuẩn SRS, bao gồm các phần: kiểm soát tài liệu, lịch sử phiên bản, phạm vi, thuật ngữ, yêu cầu về giao diện bên ngoài, định nghĩa biến Cloud (Cloud Variable), quy tắc nghiệp vụ, yêu cầu chức năng và các kịch bản nghiệm thu. Ngoài ra, AI còn giúp tách biệt trọng tâm hiện tại là tính năng chống trộm khỏi những ý tưởng cũ hoặc kém phù hợp, đồng thời hướng dẫn phân tách hệ thống thành các mô-đun rõ ràng hơn như: điều khiển chế độ bảo mật, chấm điểm xâm nhập, xử lý thiết bị tin cậy, thông báo qua Telegram, chụp ảnh từ camera, lọc cảnh báo giả/vật nuôi và cảnh báo sớm qua WiFi/MAC.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Sau buổi review tuần 7, tôi nhận ra tài liệu ban đầu của dự án IoT bị phân mảnh: có phần thiên về phần cứng, có phần chỉ ghi ý tưởng cảnh báo, có phần chưa xác định rõ phạm vi hệ thống. Từ môn SWR — Software Requirements, môn yêu cầu phần mềm — tôi hiểu rằng một hệ thống nghiêm túc cần có tài liệu đặc tả yêu cầu rõ ràng để tránh việc AI agent hiểu sai ngữ cảnh, tự thêm module không phù hợp hoặc triển khai lệch mục tiêu.
+Creative Synthesis: Tôi kết hợp kiến thức từ SWR với dự án IOT102 để tái cấu trúc lại hệ thống thành một SRS — Software Requirements Specification, tài liệu đặc tả yêu cầu phần mềm — có kiểm soát. Thay vì giữ các ghi chú rời rạc, tôi cùng AI phân rã lại hệ thống thành phạm vi dự án, lịch sử phiên bản, quyết định loại bỏ khỏi phạm vi, quy tắc cho AI agent, FR — Functional Requirement, yêu cầu chức năng, BR — Business Rule, quy tắc nghiệp vụ, Cloud Variables — biến Arduino Cloud, và Acceptance Scenarios — kịch bản chấp nhận.
+Decision Ownership: Tôi quyết định không chỉ viết lại tài liệu cho chuyên nghiệp hơn, mà còn xem lại các tài liệu ban đầu để đánh giá ý tưởng nào còn hợp lý sau review tuần 7. AI hỗ trợ tôi đặt câu hỏi, phân rã và tổ chức lại tài liệu, nhưng tôi là người kiểm soát phạm vi cuối cùng, quyết định phần nào giữ lại, phần nào loại bỏ, và biến SRS thành nguồn sự thật chính cho cả con người lẫn AI agent.</t>
+  </si>
+  <si>
+    <t>Decomposition / Pattern Recognition</t>
+  </si>
+  <si>
+    <t>005</t>
+  </si>
+  <si>
+    <t>Context Oversimplification / Requirement Misinterpretation</t>
+  </si>
+  <si>
+    <t>AI ban đầu có xu hướng hiểu công việc này chỉ là viết lại hoặc chuẩn hóa tài liệu SRS cho chuyên nghiệp hơn. AI tập trung vào việc sắp xếp lại nội dung thành các mục như phạm vi, thuật ngữ, FR, BR, Cloud Variables và Acceptance Scenarios.</t>
+  </si>
+  <si>
+    <t>Thực tế, sau buổi review tuần 7, tôi không chỉ muốn viết lại tài liệu cho đẹp hơn. Tôi cần đánh giá lại toàn bộ các tài liệu ban đầu để xem ý tưởng nào còn hợp lý, ý tưởng nào đã lệch khỏi hướng chống trộm hiện tại, và phần nào cần loại bỏ khỏi phạm vi. Đây là quá trình reassessment — đánh giá lại yêu cầu — chứ không chỉ là formatting — định dạng lại tài liệu.</t>
+  </si>
+  <si>
+    <t>Tôi phát hiện vấn đề này khi đối chiếu phản hồi sau review tuần 7 với các tài liệu cũ của dự án. Tôi nhận ra nếu chỉ để AI “chuẩn hóa SRS”, AI có thể giữ lại hoặc sắp xếp lại cả những ý tưởng cũ không còn phù hợp. Từ kiến thức môn SWR, tôi hiểu rằng tài liệu đặc tả yêu cầu phải làm rõ hệ thống làm gì, không làm gì, và phải trở thành nguồn sự thật chính cho cả người làm lẫn AI agent.</t>
+  </si>
+  <si>
+    <t>Tôi yêu cầu AI chỉnh lại entry 005 để nhấn mạnh rằng công việc này là đánh giá lại tài liệu sau review tuần 7, kiểm tra các ý tưởng cũ, kiểm soát phạm vi, loại bỏ phần không còn phù hợp, và xây dựng lại SRS như nguồn sự thật chính. Tôi cũng bổ sung phần Decision Ownership để thể hiện tôi là người quyết định cuối cùng, không để AI tự giữ hoặc thêm module ngoài phạm vi.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1qZoiVEuj7g2FTk-8AaJ4h86rMil4HBW7/view?usp=sharing</t>
+  </si>
 </sst>
 </file>
 
@@ -743,7 +778,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -859,6 +894,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -910,11 +963,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -987,13 +1042,19 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1003,16 +1064,27 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink 2" xfId="3" xr:uid="{0F39DE54-76A4-4BC0-9C10-0A0354B8E567}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{4A3D43EC-A804-43A7-AE7E-A9BE9D3942BF}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1323,14 +1395,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="18.75">
       <c r="A3" s="1" t="s">
@@ -1342,7 +1414,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1350,7 +1422,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1358,7 +1430,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1366,7 +1438,7 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="18.75">
@@ -1379,7 +1451,7 @@
         <v>7</v>
       </c>
       <c r="C10">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1387,7 +1459,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1396,7 +1468,7 @@
       </c>
       <c r="C12" s="4">
         <f>C11/C10</f>
-        <v>0.1</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>10</v>
@@ -1431,16 +1503,16 @@
     </row>
     <row r="17" spans="1:4" ht="60">
       <c r="A17" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="B17" s="19" t="s">
         <v>107</v>
-      </c>
-      <c r="B17" s="19" t="s">
-        <v>108</v>
       </c>
       <c r="C17" s="18" t="s">
         <v>18</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="60">
@@ -1448,55 +1520,55 @@
         <v>17</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C18" s="18" t="s">
         <v>19</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="60">
       <c r="A19" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="B19" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="B19" s="21" t="s">
+      <c r="C19" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="D19" s="21" t="s">
         <v>114</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="60">
       <c r="A20" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="B20" s="21" t="s">
         <v>116</v>
-      </c>
-      <c r="B20" s="21" t="s">
-        <v>117</v>
       </c>
       <c r="C20" s="18" t="s">
         <v>18</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="60">
       <c r="A21" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="B21" s="21" t="s">
         <v>119</v>
-      </c>
-      <c r="B21" s="21" t="s">
-        <v>120</v>
       </c>
       <c r="C21" s="22" t="s">
         <v>19</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -1507,62 +1579,62 @@
     </row>
     <row r="23" spans="1:4" ht="18.75">
       <c r="A23" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="C24" s="6" t="s">
         <v>23</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="8">
+        <v>2</v>
+      </c>
+      <c r="C25" s="9" t="s">
         <v>25</v>
-      </c>
-      <c r="B25" s="8">
-        <v>1</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B26" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B27" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B28" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1589,168 +1661,184 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
+      <c r="A1" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
       <c r="A2" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
+        <v>30</v>
+      </c>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
     </row>
     <row r="3" spans="1:8" ht="40.15" customHeight="1">
       <c r="A3" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>38</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="285">
       <c r="A4" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>41</v>
-      </c>
       <c r="C4" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D4" s="23" t="s">
+        <v>121</v>
+      </c>
+      <c r="E4" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="F4" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="H4" s="24" t="s">
         <v>125</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="H4" s="24" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="409.5">
       <c r="A5" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D5" s="28" t="s">
+        <v>126</v>
+      </c>
+      <c r="E5" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="E5" s="28" t="s">
+      <c r="F5" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>130</v>
-      </c>
       <c r="H5" s="24" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="150">
       <c r="A6" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C6" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="D6" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="D6" s="27" t="s">
+      <c r="E6" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="E6" s="27" t="s">
+      <c r="F6" s="28" t="s">
         <v>140</v>
       </c>
-      <c r="F6" s="28" t="s">
+      <c r="G6" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="G6" s="36" t="s">
-        <v>142</v>
-      </c>
       <c r="H6" s="24" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="165">
       <c r="A7" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D7" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="E7" s="27" t="s">
         <v>143</v>
       </c>
-      <c r="E7" s="27" t="s">
+      <c r="F7" s="28" t="s">
         <v>144</v>
       </c>
-      <c r="F7" s="28" t="s">
+      <c r="G7" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="G7" s="37" t="s">
-        <v>146</v>
-      </c>
       <c r="H7" s="24" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="409.5">
+      <c r="A8" s="42" t="s">
+        <v>154</v>
+      </c>
+      <c r="B8" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="C8" s="40" t="s">
+        <v>153</v>
+      </c>
+      <c r="D8" s="38" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="79.900000000000006" customHeight="1">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
+      <c r="E8" s="39" t="s">
+        <v>150</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="H8" s="24" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="79.900000000000006" customHeight="1">
       <c r="A9" s="7"/>
@@ -1943,6 +2031,7 @@
     <hyperlink ref="H5" r:id="rId2" xr:uid="{606E17E0-F9F6-478C-864C-0CD01FABBA13}"/>
     <hyperlink ref="H6" r:id="rId3" xr:uid="{772CBA12-EA29-48AD-8404-9EB11CE486BD}"/>
     <hyperlink ref="H7" r:id="rId4" xr:uid="{8C1F347D-6B85-4606-94B2-7F35A39F8D90}"/>
+    <hyperlink ref="H8" r:id="rId5" xr:uid="{2C82715D-BEDA-4988-81FF-86A61232C17B}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1959,74 +2048,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="33" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="40.15" customHeight="1">
       <c r="A3" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="315">
       <c r="A4" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B4" s="27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C4" s="27" t="s">
+        <v>130</v>
+      </c>
+      <c r="D4" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="E4" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="E4" s="26" t="s">
+      <c r="F4" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="F4" s="7" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="30">
-      <c r="A5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
+    </row>
+    <row r="5" spans="1:6" ht="195">
+      <c r="A5" s="42" t="s">
+        <v>154</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="6" spans="1:6" ht="60" customHeight="1">
       <c r="A6" s="7"/>
@@ -2182,73 +2281,73 @@
     </row>
     <row r="30" spans="1:6" ht="18.75">
       <c r="A30" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="C31" s="10" t="s">
         <v>55</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="30">
       <c r="A32" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B32" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" s="7" t="s">
         <v>57</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="30">
       <c r="A33" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B33" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="C33" s="7" t="s">
         <v>60</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="30">
       <c r="A34" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B34" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="C34" s="7" t="s">
         <v>63</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="30">
       <c r="A35" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="C35" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="45">
       <c r="A36" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B36" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="C36" s="7" t="s">
         <v>69</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -2272,221 +2371,221 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="37" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="35" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
     </row>
     <row r="4" spans="1:4" ht="18.75">
       <c r="A4" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="C5" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="11" t="s">
         <v>76</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>79</v>
-      </c>
       <c r="C6" s="29" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D6" s="13"/>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B7" s="13" t="s">
-        <v>82</v>
-      </c>
       <c r="C7" s="29" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D7" s="13"/>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="B8" s="13" t="s">
-        <v>84</v>
-      </c>
       <c r="C8" s="29" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D8" s="13"/>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="13" t="s">
-        <v>86</v>
-      </c>
       <c r="C9" s="29" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D9" s="13"/>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="B10" s="13" t="s">
-        <v>88</v>
-      </c>
       <c r="C10" s="29" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D10" s="13"/>
     </row>
     <row r="12" spans="1:4" ht="18.75">
       <c r="A12" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="C13" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>76</v>
-      </c>
       <c r="D13" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D14" s="13"/>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D15" s="13"/>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D16" s="13"/>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D17" s="13"/>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D18" s="13"/>
     </row>
     <row r="20" spans="1:4" ht="15.75">
       <c r="A20" s="14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="18.75">
       <c r="A25" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="60">
       <c r="A27" s="17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B27" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="C27" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="D27" s="10" t="s">
         <v>102</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -2494,7 +2593,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -2502,7 +2601,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>

</xml_diff>